<commit_message>
Complete theoretical background and procedure for L11
</commit_message>
<xml_diff>
--- a/Lab B/Lab11/L11_part_2.xlsx
+++ b/Lab B/Lab11/L11_part_2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teva\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\School\openu-courses\Lab B\Lab11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97FA3B85-2D5B-4E8B-BE9D-791FF64EFF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B616617-E904-4FA0-8190-82BA2AD98157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{16D01DD9-B812-4753-A392-552EDD7F64AD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{16D01DD9-B812-4753-A392-552EDD7F64AD}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -56,7 +53,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -102,9 +99,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -142,7 +139,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -248,7 +245,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -390,7 +387,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -398,511 +395,512 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AADC06AA-FB7D-4BEF-A219-59AF6E7C1E90}">
-  <dimension ref="J3:L44"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="11" max="11" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="K3" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="L3" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>0</v>
       </c>
-      <c r="K4">
+      <c r="B2">
         <v>1.2</v>
       </c>
-      <c r="L4">
-        <f>K4/10</f>
+      <c r="C2">
+        <f>B2/10</f>
         <v>0.12</v>
       </c>
     </row>
-    <row r="5" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J5">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="K5">
+      <c r="B3">
         <v>1.2</v>
       </c>
-      <c r="L5">
-        <f t="shared" ref="L5:L44" si="0">K5/10</f>
+      <c r="C3">
+        <f t="shared" ref="C3:C42" si="0">B3/10</f>
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J6">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>4</v>
       </c>
-      <c r="K6">
+      <c r="B4">
         <v>1.2</v>
       </c>
-      <c r="L6">
+      <c r="C4">
         <f t="shared" si="0"/>
         <v>0.12</v>
       </c>
     </row>
-    <row r="7" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J7">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>6</v>
       </c>
-      <c r="K7">
+      <c r="B5">
         <v>1.2</v>
       </c>
-      <c r="L7">
+      <c r="C5">
         <f t="shared" si="0"/>
         <v>0.12</v>
       </c>
     </row>
-    <row r="8" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J8">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>8</v>
       </c>
-      <c r="K8">
+      <c r="B6">
         <v>1.2</v>
       </c>
-      <c r="L8">
+      <c r="C6">
         <f t="shared" si="0"/>
         <v>0.12</v>
       </c>
     </row>
-    <row r="9" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J9">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>10</v>
       </c>
-      <c r="K9">
+      <c r="B7">
         <v>1.2</v>
       </c>
-      <c r="L9">
+      <c r="C7">
         <f t="shared" si="0"/>
         <v>0.12</v>
       </c>
     </row>
-    <row r="10" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J10">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>12</v>
       </c>
-      <c r="K10">
+      <c r="B8">
         <v>1.25</v>
       </c>
-      <c r="L10">
+      <c r="C8">
         <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
     </row>
-    <row r="11" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J11">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>14</v>
       </c>
-      <c r="K11">
+      <c r="B9">
         <v>1.4</v>
       </c>
-      <c r="L11">
+      <c r="C9">
         <f t="shared" si="0"/>
         <v>0.13999999999999999</v>
       </c>
     </row>
-    <row r="12" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J12">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
         <v>16</v>
       </c>
-      <c r="K12">
+      <c r="B10">
         <v>1.5</v>
       </c>
-      <c r="L12">
+      <c r="C10">
         <f t="shared" si="0"/>
         <v>0.15</v>
       </c>
     </row>
-    <row r="13" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J13">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
         <v>18</v>
       </c>
-      <c r="K13">
+      <c r="B11">
         <v>1.6</v>
       </c>
-      <c r="L13">
+      <c r="C11">
         <f t="shared" si="0"/>
         <v>0.16</v>
       </c>
     </row>
-    <row r="14" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J14">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
         <v>20</v>
       </c>
-      <c r="K14">
+      <c r="B12">
         <v>1.4</v>
       </c>
-      <c r="L14">
+      <c r="C12">
         <f t="shared" si="0"/>
         <v>0.13999999999999999</v>
       </c>
     </row>
-    <row r="15" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J15">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13">
         <v>22</v>
       </c>
-      <c r="K15">
+      <c r="B13">
         <v>1.3</v>
       </c>
-      <c r="L15">
+      <c r="C13">
         <f t="shared" si="0"/>
         <v>0.13</v>
       </c>
     </row>
-    <row r="16" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J16">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
         <v>24</v>
       </c>
-      <c r="K16">
+      <c r="B14">
         <v>1.3</v>
       </c>
-      <c r="L16">
+      <c r="C14">
         <f t="shared" si="0"/>
         <v>0.13</v>
       </c>
     </row>
-    <row r="17" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J17">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15">
         <v>26</v>
       </c>
-      <c r="K17">
+      <c r="B15">
         <v>1.5</v>
       </c>
-      <c r="L17">
+      <c r="C15">
         <f t="shared" si="0"/>
         <v>0.15</v>
       </c>
     </row>
-    <row r="18" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J18">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
         <v>28</v>
       </c>
-      <c r="K18">
+      <c r="B16">
         <v>1.8</v>
       </c>
-      <c r="L18">
+      <c r="C16">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
-    <row r="19" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J19">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17">
         <v>30</v>
       </c>
-      <c r="K19">
+      <c r="B17">
         <v>1.8</v>
       </c>
-      <c r="L19">
+      <c r="C17">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
-    <row r="20" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J20">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
         <v>32</v>
       </c>
-      <c r="K20">
+      <c r="B18">
         <v>1.5</v>
       </c>
-      <c r="L20">
+      <c r="C18">
         <f t="shared" si="0"/>
         <v>0.15</v>
       </c>
     </row>
-    <row r="21" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J21">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19">
         <v>34</v>
       </c>
-      <c r="K21">
+      <c r="B19">
         <v>1.3</v>
       </c>
-      <c r="L21">
+      <c r="C19">
         <f t="shared" si="0"/>
         <v>0.13</v>
       </c>
     </row>
-    <row r="22" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J22">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20">
         <v>36</v>
       </c>
-      <c r="K22">
+      <c r="B20">
         <v>1.4</v>
       </c>
-      <c r="L22">
+      <c r="C20">
         <f t="shared" si="0"/>
         <v>0.13999999999999999</v>
       </c>
     </row>
-    <row r="23" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J23">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21">
         <v>38</v>
       </c>
-      <c r="K23">
+      <c r="B21">
         <v>1.8</v>
       </c>
-      <c r="L23">
+      <c r="C21">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
-    <row r="24" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J24">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22">
         <v>40</v>
       </c>
-      <c r="K24">
+      <c r="B22">
         <v>2.1</v>
       </c>
-      <c r="L24">
+      <c r="C22">
         <f t="shared" si="0"/>
         <v>0.21000000000000002</v>
       </c>
     </row>
-    <row r="25" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
         <v>42</v>
       </c>
-      <c r="K25">
+      <c r="B23">
         <v>2</v>
       </c>
-      <c r="L25">
+      <c r="C23">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
     </row>
-    <row r="26" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J26">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24">
         <v>44</v>
       </c>
-      <c r="K26">
+      <c r="B24">
         <v>1.6</v>
       </c>
-      <c r="L26">
+      <c r="C24">
         <f t="shared" si="0"/>
         <v>0.16</v>
       </c>
     </row>
-    <row r="27" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J27">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
         <v>46</v>
       </c>
-      <c r="K27">
+      <c r="B25">
         <v>1.4</v>
       </c>
-      <c r="L27">
+      <c r="C25">
         <f t="shared" si="0"/>
         <v>0.13999999999999999</v>
       </c>
     </row>
-    <row r="28" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J28">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
         <v>48</v>
       </c>
-      <c r="K28">
+      <c r="B26">
         <v>1.4</v>
       </c>
-      <c r="L28">
+      <c r="C26">
         <f t="shared" si="0"/>
         <v>0.13999999999999999</v>
       </c>
     </row>
-    <row r="29" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J29">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27">
         <v>50</v>
       </c>
-      <c r="K29">
+      <c r="B27">
         <v>1.8</v>
       </c>
-      <c r="L29">
+      <c r="C27">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
-    <row r="30" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J30">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
         <v>52</v>
       </c>
-      <c r="K30">
+      <c r="B28">
         <v>2.2000000000000002</v>
       </c>
-      <c r="L30">
+      <c r="C28">
         <f t="shared" si="0"/>
         <v>0.22000000000000003</v>
       </c>
     </row>
-    <row r="31" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J31">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
         <v>54</v>
       </c>
-      <c r="K31">
+      <c r="B29">
         <v>2.2000000000000002</v>
       </c>
-      <c r="L31">
+      <c r="C29">
         <f t="shared" si="0"/>
         <v>0.22000000000000003</v>
       </c>
     </row>
-    <row r="32" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J32">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30">
         <v>56</v>
       </c>
-      <c r="K32">
+      <c r="B30">
         <v>1.9</v>
       </c>
-      <c r="L32">
+      <c r="C30">
         <f t="shared" si="0"/>
         <v>0.19</v>
       </c>
     </row>
-    <row r="33" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J33">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31">
         <v>58</v>
       </c>
-      <c r="K33">
+      <c r="B31">
         <v>1.6</v>
       </c>
-      <c r="L33">
+      <c r="C31">
         <f t="shared" si="0"/>
         <v>0.16</v>
       </c>
     </row>
-    <row r="34" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J34">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32">
         <v>60</v>
       </c>
-      <c r="K34">
+      <c r="B32">
         <v>1.5</v>
       </c>
-      <c r="L34">
+      <c r="C32">
         <f t="shared" si="0"/>
         <v>0.15</v>
       </c>
     </row>
-    <row r="35" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33">
         <v>62</v>
       </c>
-      <c r="K35">
+      <c r="B33">
         <v>1.6</v>
       </c>
-      <c r="L35">
+      <c r="C33">
         <f t="shared" si="0"/>
         <v>0.16</v>
       </c>
     </row>
-    <row r="36" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J36">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34">
         <v>64</v>
       </c>
-      <c r="K36">
+      <c r="B34">
         <v>2</v>
       </c>
-      <c r="L36">
+      <c r="C34">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
     </row>
-    <row r="37" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J37">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35">
         <v>66</v>
       </c>
-      <c r="K37">
+      <c r="B35">
         <v>2.2999999999999998</v>
       </c>
-      <c r="L37">
+      <c r="C35">
         <f t="shared" si="0"/>
         <v>0.22999999999999998</v>
       </c>
     </row>
-    <row r="38" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J38">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36">
         <v>68</v>
       </c>
-      <c r="K38">
+      <c r="B36">
         <v>2.2999999999999998</v>
       </c>
-      <c r="L38">
+      <c r="C36">
         <f t="shared" si="0"/>
         <v>0.22999999999999998</v>
       </c>
     </row>
-    <row r="39" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J39">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
         <v>70</v>
       </c>
-      <c r="K39">
+      <c r="B37">
         <v>2</v>
       </c>
-      <c r="L39">
+      <c r="C37">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
     </row>
-    <row r="40" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J40">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38">
         <v>72</v>
       </c>
-      <c r="K40">
+      <c r="B38">
         <v>1.8</v>
       </c>
-      <c r="L40">
+      <c r="C38">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
-    <row r="41" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J41">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39">
         <v>74</v>
       </c>
-      <c r="K41">
+      <c r="B39">
         <v>1.8</v>
       </c>
-      <c r="L41">
+      <c r="C39">
         <f t="shared" si="0"/>
         <v>0.18</v>
       </c>
     </row>
-    <row r="42" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J42">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40">
         <v>76</v>
       </c>
-      <c r="K42">
+      <c r="B40">
         <v>2.1</v>
       </c>
-      <c r="L42">
+      <c r="C40">
         <f t="shared" si="0"/>
         <v>0.21000000000000002</v>
       </c>
     </row>
-    <row r="43" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J43">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41">
         <v>78</v>
       </c>
-      <c r="K43">
+      <c r="B41">
         <v>2.4</v>
       </c>
-      <c r="L43">
+      <c r="C41">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
     </row>
-    <row r="44" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J44">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42">
         <v>80</v>
       </c>
-      <c r="K44">
+      <c r="B42">
         <v>2.4</v>
       </c>
-      <c r="L44">
+      <c r="C42">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>

</xml_diff>